<commit_message>
Show F rows with zero values and CV; rename Spending Analysis; update Allocation Input Form
</commit_message>
<xml_diff>
--- a/Allocation Input Form.xlsx
+++ b/Allocation Input Form.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29713"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mszek\OneDrive\Desktop\2019SHS\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mszekely\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{332CB63C-07C6-4504-98C1-789DD4527DF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C6D9FEED-3418-4D94-BBE9-D9ACE0A64CE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-12615" yWindow="-21720" windowWidth="51840" windowHeight="21840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2490" yWindow="0" windowWidth="25170" windowHeight="21705" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Spending Estimates" sheetId="1" r:id="rId1"/>
@@ -2230,7 +2230,8 @@
   <dimension ref="A1:D303"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="50" customWidth="1"/>
+    <col min="1" max="1" width="50" customWidth="1"/>
+    <col min="2" max="2" width="59.42578125" customWidth="1"/>
     <col min="3" max="3" width="26.5703125" style="1" customWidth="1"/>
     <col min="4" max="4" width="23.28515625" style="1" customWidth="1"/>
   </cols>
@@ -2275,11 +2276,9 @@
         <v>6</v>
       </c>
       <c r="C5" s="4">
-        <v>0.7</v>
-      </c>
-      <c r="D5" s="5">
-        <v>4</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="D5" s="5"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
@@ -2289,7 +2288,7 @@
         <v>8</v>
       </c>
       <c r="C6" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D6" s="5">
         <v>4</v>
@@ -2303,10 +2302,10 @@
         <v>10</v>
       </c>
       <c r="C7" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D7" s="5">
-        <v>4</v>
+        <v>4.0011997600479905</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -2317,7 +2316,7 @@
         <v>12</v>
       </c>
       <c r="C8" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D8" s="5">
         <v>4</v>
@@ -2331,7 +2330,7 @@
         <v>14</v>
       </c>
       <c r="C9" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D9" s="5">
         <v>4</v>
@@ -2345,7 +2344,7 @@
         <v>16</v>
       </c>
       <c r="C10" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D10" s="5">
         <v>4</v>
@@ -2359,7 +2358,7 @@
         <v>18</v>
       </c>
       <c r="C11" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D11" s="5">
         <v>4</v>
@@ -2373,7 +2372,7 @@
         <v>20</v>
       </c>
       <c r="C12" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D12" s="5">
         <v>4</v>
@@ -2387,7 +2386,7 @@
         <v>22</v>
       </c>
       <c r="C13" s="4">
-        <v>0.65</v>
+        <v>0</v>
       </c>
       <c r="D13" s="5">
         <v>4</v>
@@ -2401,7 +2400,7 @@
         <v>24</v>
       </c>
       <c r="C14" s="4">
-        <v>0.65</v>
+        <v>0</v>
       </c>
       <c r="D14" s="5">
         <v>4</v>
@@ -2415,7 +2414,7 @@
         <v>26</v>
       </c>
       <c r="C15" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D15" s="5">
         <v>4</v>
@@ -2429,7 +2428,7 @@
         <v>28</v>
       </c>
       <c r="C16" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D16" s="5">
         <v>4</v>
@@ -2443,7 +2442,7 @@
         <v>30</v>
       </c>
       <c r="C17" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D17" s="5">
         <v>4</v>
@@ -2457,7 +2456,7 @@
         <v>32</v>
       </c>
       <c r="C18" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D18" s="5">
         <v>4</v>
@@ -2471,7 +2470,7 @@
         <v>34</v>
       </c>
       <c r="C19" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D19" s="5">
         <v>4</v>
@@ -2485,7 +2484,7 @@
         <v>36</v>
       </c>
       <c r="C20" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D20" s="5">
         <v>4</v>
@@ -2499,7 +2498,7 @@
         <v>38</v>
       </c>
       <c r="C21" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D21" s="5">
         <v>4</v>
@@ -2513,7 +2512,7 @@
         <v>40</v>
       </c>
       <c r="C22" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D22" s="5">
         <v>4</v>
@@ -2527,7 +2526,7 @@
         <v>42</v>
       </c>
       <c r="C23" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D23" s="5">
         <v>4</v>
@@ -2541,7 +2540,7 @@
         <v>44</v>
       </c>
       <c r="C24" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D24" s="5">
         <v>4</v>
@@ -2555,7 +2554,7 @@
         <v>46</v>
       </c>
       <c r="C25" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D25" s="5">
         <v>4</v>
@@ -2569,7 +2568,7 @@
         <v>48</v>
       </c>
       <c r="C26" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D26" s="5">
         <v>4</v>
@@ -2583,7 +2582,7 @@
         <v>50</v>
       </c>
       <c r="C27" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D27" s="5">
         <v>4</v>
@@ -2597,7 +2596,7 @@
         <v>52</v>
       </c>
       <c r="C28" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D28" s="5">
         <v>4</v>
@@ -2611,7 +2610,7 @@
         <v>54</v>
       </c>
       <c r="C29" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D29" s="5">
         <v>4</v>
@@ -2625,7 +2624,7 @@
         <v>56</v>
       </c>
       <c r="C30" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D30" s="5">
         <v>4</v>
@@ -2639,7 +2638,7 @@
         <v>58</v>
       </c>
       <c r="C31" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D31" s="5">
         <v>4</v>
@@ -2653,7 +2652,7 @@
         <v>60</v>
       </c>
       <c r="C32" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D32" s="5">
         <v>4</v>
@@ -2667,7 +2666,7 @@
         <v>62</v>
       </c>
       <c r="C33" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D33" s="5">
         <v>4</v>
@@ -2681,7 +2680,7 @@
         <v>64</v>
       </c>
       <c r="C34" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D34" s="5">
         <v>4</v>
@@ -2695,7 +2694,7 @@
         <v>66</v>
       </c>
       <c r="C35" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D35" s="5">
         <v>4</v>
@@ -2709,7 +2708,7 @@
         <v>68</v>
       </c>
       <c r="C36" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D36" s="5">
         <v>4</v>
@@ -2723,7 +2722,7 @@
         <v>70</v>
       </c>
       <c r="C37" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D37" s="5">
         <v>4</v>
@@ -2737,7 +2736,7 @@
         <v>72</v>
       </c>
       <c r="C38" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D38" s="5">
         <v>4</v>
@@ -2751,7 +2750,7 @@
         <v>74</v>
       </c>
       <c r="C39" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D39" s="5">
         <v>4</v>
@@ -2765,7 +2764,7 @@
         <v>76</v>
       </c>
       <c r="C40" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D40" s="5">
         <v>4</v>
@@ -2779,7 +2778,7 @@
         <v>78</v>
       </c>
       <c r="C41" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D41" s="5">
         <v>4</v>
@@ -2793,7 +2792,7 @@
         <v>80</v>
       </c>
       <c r="C42" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D42" s="5">
         <v>4</v>
@@ -2807,7 +2806,7 @@
         <v>82</v>
       </c>
       <c r="C43" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D43" s="5">
         <v>4</v>
@@ -2821,7 +2820,7 @@
         <v>84</v>
       </c>
       <c r="C44" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D44" s="5">
         <v>4</v>
@@ -2835,7 +2834,7 @@
         <v>86</v>
       </c>
       <c r="C45" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D45" s="5">
         <v>4</v>
@@ -2849,7 +2848,7 @@
         <v>88</v>
       </c>
       <c r="C46" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D46" s="5">
         <v>4</v>
@@ -2863,7 +2862,7 @@
         <v>90</v>
       </c>
       <c r="C47" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D47" s="5">
         <v>4</v>
@@ -2877,7 +2876,7 @@
         <v>92</v>
       </c>
       <c r="C48" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D48" s="5">
         <v>4</v>
@@ -2891,7 +2890,7 @@
         <v>94</v>
       </c>
       <c r="C49" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D49" s="5">
         <v>4</v>
@@ -2905,7 +2904,7 @@
         <v>96</v>
       </c>
       <c r="C50" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D50" s="5">
         <v>4</v>
@@ -2919,7 +2918,7 @@
         <v>98</v>
       </c>
       <c r="C51" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D51" s="5">
         <v>4</v>
@@ -2933,7 +2932,7 @@
         <v>100</v>
       </c>
       <c r="C52" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D52" s="5">
         <v>4</v>
@@ -2947,7 +2946,7 @@
         <v>102</v>
       </c>
       <c r="C53" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D53" s="5">
         <v>4</v>
@@ -2961,7 +2960,7 @@
         <v>104</v>
       </c>
       <c r="C54" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D54" s="5">
         <v>4</v>
@@ -2975,10 +2974,10 @@
         <v>106</v>
       </c>
       <c r="C55" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D55" s="5">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
@@ -2989,10 +2988,10 @@
         <v>108</v>
       </c>
       <c r="C56" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D56" s="5">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
@@ -3003,10 +3002,10 @@
         <v>110</v>
       </c>
       <c r="C57" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D57" s="5">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
@@ -3017,10 +3016,10 @@
         <v>112</v>
       </c>
       <c r="C58" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D58" s="5">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
@@ -3031,10 +3030,10 @@
         <v>114</v>
       </c>
       <c r="C59" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D59" s="5">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
@@ -3045,10 +3044,10 @@
         <v>116</v>
       </c>
       <c r="C60" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D60" s="5">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
@@ -3059,10 +3058,10 @@
         <v>118</v>
       </c>
       <c r="C61" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D61" s="5">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
@@ -3073,10 +3072,10 @@
         <v>120</v>
       </c>
       <c r="C62" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D62" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
@@ -3087,10 +3086,10 @@
         <v>122</v>
       </c>
       <c r="C63" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D63" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
@@ -3101,10 +3100,10 @@
         <v>124</v>
       </c>
       <c r="C64" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D64" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
@@ -3115,10 +3114,10 @@
         <v>126</v>
       </c>
       <c r="C65" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D65" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
@@ -3129,10 +3128,10 @@
         <v>128</v>
       </c>
       <c r="C66" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D66" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
@@ -3143,10 +3142,10 @@
         <v>130</v>
       </c>
       <c r="C67" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D67" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
@@ -3157,10 +3156,10 @@
         <v>132</v>
       </c>
       <c r="C68" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D68" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
@@ -3171,10 +3170,10 @@
         <v>134</v>
       </c>
       <c r="C69" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D69" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
@@ -3185,10 +3184,10 @@
         <v>136</v>
       </c>
       <c r="C70" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D70" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
@@ -3199,10 +3198,10 @@
         <v>138</v>
       </c>
       <c r="C71" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D71" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
@@ -3213,10 +3212,10 @@
         <v>140</v>
       </c>
       <c r="C72" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D72" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
@@ -3227,10 +3226,10 @@
         <v>142</v>
       </c>
       <c r="C73" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D73" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
@@ -3241,10 +3240,10 @@
         <v>144</v>
       </c>
       <c r="C74" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D74" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
@@ -3255,10 +3254,10 @@
         <v>146</v>
       </c>
       <c r="C75" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D75" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
@@ -3269,10 +3268,10 @@
         <v>148</v>
       </c>
       <c r="C76" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D76" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
@@ -3283,10 +3282,10 @@
         <v>150</v>
       </c>
       <c r="C77" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D77" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
@@ -3297,10 +3296,10 @@
         <v>152</v>
       </c>
       <c r="C78" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D78" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
@@ -3311,10 +3310,10 @@
         <v>154</v>
       </c>
       <c r="C79" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D79" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">
@@ -3325,10 +3324,10 @@
         <v>156</v>
       </c>
       <c r="C80" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D80" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
@@ -3339,10 +3338,10 @@
         <v>158</v>
       </c>
       <c r="C81" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D81" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
@@ -3353,10 +3352,10 @@
         <v>160</v>
       </c>
       <c r="C82" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D82" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
@@ -3367,10 +3366,10 @@
         <v>162</v>
       </c>
       <c r="C83" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D83" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
@@ -3381,10 +3380,10 @@
         <v>164</v>
       </c>
       <c r="C84" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D84" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
@@ -3395,10 +3394,10 @@
         <v>166</v>
       </c>
       <c r="C85" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D85" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
@@ -3409,10 +3408,10 @@
         <v>168</v>
       </c>
       <c r="C86" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D86" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
@@ -3423,10 +3422,10 @@
         <v>170</v>
       </c>
       <c r="C87" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D87" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
@@ -3437,10 +3436,10 @@
         <v>172</v>
       </c>
       <c r="C88" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D88" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
@@ -3451,10 +3450,10 @@
         <v>174</v>
       </c>
       <c r="C89" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D89" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.25">
@@ -3465,10 +3464,10 @@
         <v>176</v>
       </c>
       <c r="C90" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D90" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
@@ -3479,10 +3478,10 @@
         <v>178</v>
       </c>
       <c r="C91" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D91" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.25">
@@ -3493,10 +3492,10 @@
         <v>180</v>
       </c>
       <c r="C92" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D92" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.25">
@@ -3507,10 +3506,10 @@
         <v>182</v>
       </c>
       <c r="C93" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D93" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.25">
@@ -3521,10 +3520,10 @@
         <v>184</v>
       </c>
       <c r="C94" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D94" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.25">
@@ -3535,10 +3534,10 @@
         <v>186</v>
       </c>
       <c r="C95" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D95" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.25">
@@ -3549,10 +3548,10 @@
         <v>188</v>
       </c>
       <c r="C96" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D96" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
@@ -3563,10 +3562,10 @@
         <v>190</v>
       </c>
       <c r="C97" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D97" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
@@ -3577,10 +3576,10 @@
         <v>192</v>
       </c>
       <c r="C98" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D98" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.25">
@@ -3591,10 +3590,10 @@
         <v>194</v>
       </c>
       <c r="C99" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D99" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.25">
@@ -3605,10 +3604,10 @@
         <v>196</v>
       </c>
       <c r="C100" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D100" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.25">
@@ -3619,10 +3618,10 @@
         <v>198</v>
       </c>
       <c r="C101" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D101" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.25">
@@ -3633,10 +3632,10 @@
         <v>200</v>
       </c>
       <c r="C102" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D102" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.25">
@@ -3647,10 +3646,10 @@
         <v>202</v>
       </c>
       <c r="C103" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D103" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.25">
@@ -3661,10 +3660,10 @@
         <v>204</v>
       </c>
       <c r="C104" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D104" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.25">
@@ -3675,10 +3674,10 @@
         <v>206</v>
       </c>
       <c r="C105" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D105" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.25">
@@ -3689,10 +3688,10 @@
         <v>208</v>
       </c>
       <c r="C106" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D106" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.25">
@@ -3703,10 +3702,10 @@
         <v>210</v>
       </c>
       <c r="C107" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D107" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.25">
@@ -3717,10 +3716,10 @@
         <v>212</v>
       </c>
       <c r="C108" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D108" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.25">
@@ -3731,10 +3730,10 @@
         <v>214</v>
       </c>
       <c r="C109" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D109" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.25">
@@ -3745,10 +3744,10 @@
         <v>216</v>
       </c>
       <c r="C110" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D110" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.25">
@@ -3759,10 +3758,10 @@
         <v>218</v>
       </c>
       <c r="C111" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D111" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.25">
@@ -3773,10 +3772,10 @@
         <v>220</v>
       </c>
       <c r="C112" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D112" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.25">
@@ -3787,10 +3786,10 @@
         <v>222</v>
       </c>
       <c r="C113" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D113" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.25">
@@ -3801,10 +3800,10 @@
         <v>224</v>
       </c>
       <c r="C114" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D114" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.25">
@@ -3815,10 +3814,10 @@
         <v>226</v>
       </c>
       <c r="C115" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D115" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.25">
@@ -3829,10 +3828,10 @@
         <v>228</v>
       </c>
       <c r="C116" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D116" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.25">
@@ -3843,10 +3842,10 @@
         <v>230</v>
       </c>
       <c r="C117" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D117" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.25">
@@ -3857,10 +3856,10 @@
         <v>232</v>
       </c>
       <c r="C118" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D118" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.25">
@@ -3871,10 +3870,10 @@
         <v>234</v>
       </c>
       <c r="C119" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D119" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.25">
@@ -3885,10 +3884,10 @@
         <v>236</v>
       </c>
       <c r="C120" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D120" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.25">
@@ -3899,10 +3898,10 @@
         <v>238</v>
       </c>
       <c r="C121" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D121" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.25">
@@ -3913,10 +3912,10 @@
         <v>240</v>
       </c>
       <c r="C122" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D122" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.25">
@@ -3927,10 +3926,10 @@
         <v>242</v>
       </c>
       <c r="C123" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D123" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.25">
@@ -3941,10 +3940,10 @@
         <v>244</v>
       </c>
       <c r="C124" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D124" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="125" spans="1:4" x14ac:dyDescent="0.25">
@@ -3955,10 +3954,10 @@
         <v>246</v>
       </c>
       <c r="C125" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D125" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="126" spans="1:4" x14ac:dyDescent="0.25">
@@ -3969,10 +3968,10 @@
         <v>248</v>
       </c>
       <c r="C126" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D126" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="127" spans="1:4" x14ac:dyDescent="0.25">
@@ -3983,10 +3982,10 @@
         <v>250</v>
       </c>
       <c r="C127" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D127" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="128" spans="1:4" x14ac:dyDescent="0.25">
@@ -3997,10 +3996,10 @@
         <v>252</v>
       </c>
       <c r="C128" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D128" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="129" spans="1:4" x14ac:dyDescent="0.25">
@@ -4011,10 +4010,10 @@
         <v>254</v>
       </c>
       <c r="C129" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D129" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="130" spans="1:4" x14ac:dyDescent="0.25">
@@ -4025,10 +4024,10 @@
         <v>256</v>
       </c>
       <c r="C130" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D130" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="131" spans="1:4" x14ac:dyDescent="0.25">
@@ -4039,10 +4038,10 @@
         <v>258</v>
       </c>
       <c r="C131" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D131" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="132" spans="1:4" x14ac:dyDescent="0.25">
@@ -4053,10 +4052,10 @@
         <v>260</v>
       </c>
       <c r="C132" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D132" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="133" spans="1:4" x14ac:dyDescent="0.25">
@@ -4067,10 +4066,10 @@
         <v>262</v>
       </c>
       <c r="C133" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D133" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="134" spans="1:4" x14ac:dyDescent="0.25">
@@ -4081,10 +4080,10 @@
         <v>264</v>
       </c>
       <c r="C134" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D134" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="135" spans="1:4" x14ac:dyDescent="0.25">
@@ -4095,10 +4094,10 @@
         <v>266</v>
       </c>
       <c r="C135" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D135" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="136" spans="1:4" x14ac:dyDescent="0.25">
@@ -4109,10 +4108,10 @@
         <v>268</v>
       </c>
       <c r="C136" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D136" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="137" spans="1:4" x14ac:dyDescent="0.25">
@@ -4123,10 +4122,10 @@
         <v>270</v>
       </c>
       <c r="C137" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D137" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="138" spans="1:4" x14ac:dyDescent="0.25">
@@ -4137,10 +4136,10 @@
         <v>272</v>
       </c>
       <c r="C138" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D138" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="139" spans="1:4" x14ac:dyDescent="0.25">
@@ -4151,10 +4150,10 @@
         <v>274</v>
       </c>
       <c r="C139" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D139" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="140" spans="1:4" x14ac:dyDescent="0.25">
@@ -4165,10 +4164,10 @@
         <v>276</v>
       </c>
       <c r="C140" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D140" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="141" spans="1:4" x14ac:dyDescent="0.25">
@@ -4179,10 +4178,10 @@
         <v>278</v>
       </c>
       <c r="C141" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D141" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="142" spans="1:4" x14ac:dyDescent="0.25">
@@ -4193,10 +4192,10 @@
         <v>280</v>
       </c>
       <c r="C142" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D142" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="143" spans="1:4" x14ac:dyDescent="0.25">
@@ -4207,10 +4206,10 @@
         <v>282</v>
       </c>
       <c r="C143" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D143" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="144" spans="1:4" x14ac:dyDescent="0.25">
@@ -4221,10 +4220,10 @@
         <v>284</v>
       </c>
       <c r="C144" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D144" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="145" spans="1:4" x14ac:dyDescent="0.25">
@@ -4235,10 +4234,10 @@
         <v>286</v>
       </c>
       <c r="C145" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D145" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="146" spans="1:4" x14ac:dyDescent="0.25">
@@ -4249,10 +4248,10 @@
         <v>288</v>
       </c>
       <c r="C146" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D146" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="147" spans="1:4" x14ac:dyDescent="0.25">
@@ -4263,10 +4262,10 @@
         <v>290</v>
       </c>
       <c r="C147" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D147" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="148" spans="1:4" x14ac:dyDescent="0.25">
@@ -4277,10 +4276,10 @@
         <v>292</v>
       </c>
       <c r="C148" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D148" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="149" spans="1:4" x14ac:dyDescent="0.25">
@@ -4291,10 +4290,10 @@
         <v>294</v>
       </c>
       <c r="C149" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D149" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="150" spans="1:4" x14ac:dyDescent="0.25">
@@ -4305,10 +4304,10 @@
         <v>296</v>
       </c>
       <c r="C150" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D150" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="151" spans="1:4" x14ac:dyDescent="0.25">
@@ -4319,10 +4318,10 @@
         <v>298</v>
       </c>
       <c r="C151" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D151" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="152" spans="1:4" x14ac:dyDescent="0.25">
@@ -4333,10 +4332,10 @@
         <v>300</v>
       </c>
       <c r="C152" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D152" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="153" spans="1:4" x14ac:dyDescent="0.25">
@@ -4347,10 +4346,10 @@
         <v>302</v>
       </c>
       <c r="C153" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D153" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="154" spans="1:4" x14ac:dyDescent="0.25">
@@ -4361,10 +4360,10 @@
         <v>304</v>
       </c>
       <c r="C154" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D154" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="155" spans="1:4" x14ac:dyDescent="0.25">
@@ -4375,10 +4374,10 @@
         <v>306</v>
       </c>
       <c r="C155" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D155" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="156" spans="1:4" x14ac:dyDescent="0.25">
@@ -4389,10 +4388,10 @@
         <v>308</v>
       </c>
       <c r="C156" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D156" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="157" spans="1:4" x14ac:dyDescent="0.25">
@@ -4403,10 +4402,10 @@
         <v>310</v>
       </c>
       <c r="C157" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D157" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="158" spans="1:4" x14ac:dyDescent="0.25">
@@ -4417,10 +4416,10 @@
         <v>312</v>
       </c>
       <c r="C158" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D158" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="159" spans="1:4" x14ac:dyDescent="0.25">
@@ -4431,10 +4430,10 @@
         <v>314</v>
       </c>
       <c r="C159" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D159" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="160" spans="1:4" x14ac:dyDescent="0.25">
@@ -4445,10 +4444,10 @@
         <v>316</v>
       </c>
       <c r="C160" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D160" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="161" spans="1:4" x14ac:dyDescent="0.25">
@@ -4459,10 +4458,10 @@
         <v>318</v>
       </c>
       <c r="C161" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D161" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="162" spans="1:4" x14ac:dyDescent="0.25">
@@ -4473,10 +4472,10 @@
         <v>320</v>
       </c>
       <c r="C162" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D162" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="163" spans="1:4" x14ac:dyDescent="0.25">
@@ -4490,7 +4489,7 @@
         <v>0.7</v>
       </c>
       <c r="D163" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="164" spans="1:4" x14ac:dyDescent="0.25">
@@ -4504,7 +4503,7 @@
         <v>0.7</v>
       </c>
       <c r="D164" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="165" spans="1:4" x14ac:dyDescent="0.25">
@@ -4518,7 +4517,7 @@
         <v>0.7</v>
       </c>
       <c r="D165" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="166" spans="1:4" x14ac:dyDescent="0.25">
@@ -4532,7 +4531,7 @@
         <v>0.7</v>
       </c>
       <c r="D166" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="167" spans="1:4" x14ac:dyDescent="0.25">
@@ -4546,7 +4545,7 @@
         <v>0.7</v>
       </c>
       <c r="D167" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="168" spans="1:4" x14ac:dyDescent="0.25">
@@ -4560,7 +4559,7 @@
         <v>0.7</v>
       </c>
       <c r="D168" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="169" spans="1:4" x14ac:dyDescent="0.25">
@@ -4574,7 +4573,7 @@
         <v>0.7</v>
       </c>
       <c r="D169" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="170" spans="1:4" x14ac:dyDescent="0.25">
@@ -4588,7 +4587,7 @@
         <v>0.7</v>
       </c>
       <c r="D170" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="171" spans="1:4" x14ac:dyDescent="0.25">
@@ -4602,7 +4601,7 @@
         <v>0.7</v>
       </c>
       <c r="D171" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="172" spans="1:4" x14ac:dyDescent="0.25">
@@ -4616,7 +4615,7 @@
         <v>0.7</v>
       </c>
       <c r="D172" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="173" spans="1:4" x14ac:dyDescent="0.25">
@@ -4630,7 +4629,7 @@
         <v>0.7</v>
       </c>
       <c r="D173" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="174" spans="1:4" x14ac:dyDescent="0.25">
@@ -4644,7 +4643,7 @@
         <v>0.7</v>
       </c>
       <c r="D174" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="175" spans="1:4" x14ac:dyDescent="0.25">
@@ -4658,7 +4657,7 @@
         <v>0.7</v>
       </c>
       <c r="D175" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="176" spans="1:4" x14ac:dyDescent="0.25">
@@ -4672,7 +4671,7 @@
         <v>0.7</v>
       </c>
       <c r="D176" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="177" spans="1:4" x14ac:dyDescent="0.25">
@@ -4686,7 +4685,7 @@
         <v>0.7</v>
       </c>
       <c r="D177" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="178" spans="1:4" x14ac:dyDescent="0.25">
@@ -4700,7 +4699,7 @@
         <v>0.7</v>
       </c>
       <c r="D178" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="179" spans="1:4" x14ac:dyDescent="0.25">
@@ -4714,7 +4713,7 @@
         <v>0.7</v>
       </c>
       <c r="D179" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="180" spans="1:4" x14ac:dyDescent="0.25">
@@ -4728,7 +4727,7 @@
         <v>0.7</v>
       </c>
       <c r="D180" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="181" spans="1:4" x14ac:dyDescent="0.25">
@@ -4742,7 +4741,7 @@
         <v>0.7</v>
       </c>
       <c r="D181" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="182" spans="1:4" x14ac:dyDescent="0.25">
@@ -4756,7 +4755,7 @@
         <v>0.7</v>
       </c>
       <c r="D182" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="183" spans="1:4" x14ac:dyDescent="0.25">
@@ -4770,7 +4769,7 @@
         <v>0.7</v>
       </c>
       <c r="D183" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="184" spans="1:4" x14ac:dyDescent="0.25">
@@ -5036,7 +5035,7 @@
         <v>0.7</v>
       </c>
       <c r="D202" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="203" spans="1:4" x14ac:dyDescent="0.25">
@@ -5050,7 +5049,7 @@
         <v>0.7</v>
       </c>
       <c r="D203" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="204" spans="1:4" x14ac:dyDescent="0.25">
@@ -5064,7 +5063,7 @@
         <v>0.7</v>
       </c>
       <c r="D204" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="205" spans="1:4" x14ac:dyDescent="0.25">
@@ -5078,7 +5077,7 @@
         <v>0.7</v>
       </c>
       <c r="D205" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="206" spans="1:4" x14ac:dyDescent="0.25">
@@ -5092,7 +5091,7 @@
         <v>0.7</v>
       </c>
       <c r="D206" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="207" spans="1:4" x14ac:dyDescent="0.25">
@@ -5106,7 +5105,7 @@
         <v>0.7</v>
       </c>
       <c r="D207" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="208" spans="1:4" x14ac:dyDescent="0.25">
@@ -5120,7 +5119,7 @@
         <v>0.7</v>
       </c>
       <c r="D208" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="209" spans="1:4" x14ac:dyDescent="0.25">
@@ -5134,7 +5133,7 @@
         <v>0.7</v>
       </c>
       <c r="D209" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="210" spans="1:4" x14ac:dyDescent="0.25">
@@ -5148,7 +5147,7 @@
         <v>0.7</v>
       </c>
       <c r="D210" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="211" spans="1:4" x14ac:dyDescent="0.25">
@@ -5162,7 +5161,7 @@
         <v>0.7</v>
       </c>
       <c r="D211" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="212" spans="1:4" x14ac:dyDescent="0.25">
@@ -5176,7 +5175,7 @@
         <v>0.7</v>
       </c>
       <c r="D212" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="213" spans="1:4" x14ac:dyDescent="0.25">
@@ -5190,7 +5189,7 @@
         <v>0.7</v>
       </c>
       <c r="D213" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="214" spans="1:4" x14ac:dyDescent="0.25">
@@ -5204,7 +5203,7 @@
         <v>0.7</v>
       </c>
       <c r="D214" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="215" spans="1:4" x14ac:dyDescent="0.25">
@@ -5218,7 +5217,7 @@
         <v>0.7</v>
       </c>
       <c r="D215" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="216" spans="1:4" x14ac:dyDescent="0.25">
@@ -5232,7 +5231,7 @@
         <v>0.7</v>
       </c>
       <c r="D216" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="217" spans="1:4" x14ac:dyDescent="0.25">
@@ -5243,10 +5242,10 @@
         <v>429</v>
       </c>
       <c r="C217" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D217" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="218" spans="1:4" x14ac:dyDescent="0.25">
@@ -5257,10 +5256,10 @@
         <v>431</v>
       </c>
       <c r="C218" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D218" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="219" spans="1:4" x14ac:dyDescent="0.25">
@@ -5271,10 +5270,10 @@
         <v>433</v>
       </c>
       <c r="C219" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D219" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="220" spans="1:4" x14ac:dyDescent="0.25">
@@ -5285,10 +5284,10 @@
         <v>435</v>
       </c>
       <c r="C220" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D220" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="221" spans="1:4" x14ac:dyDescent="0.25">
@@ -5299,10 +5298,10 @@
         <v>437</v>
       </c>
       <c r="C221" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D221" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="222" spans="1:4" x14ac:dyDescent="0.25">
@@ -5313,10 +5312,10 @@
         <v>439</v>
       </c>
       <c r="C222" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D222" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="223" spans="1:4" x14ac:dyDescent="0.25">
@@ -5327,10 +5326,10 @@
         <v>441</v>
       </c>
       <c r="C223" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D223" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="224" spans="1:4" x14ac:dyDescent="0.25">
@@ -5341,10 +5340,10 @@
         <v>443</v>
       </c>
       <c r="C224" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D224" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="225" spans="1:4" x14ac:dyDescent="0.25">
@@ -5355,10 +5354,10 @@
         <v>445</v>
       </c>
       <c r="C225" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D225" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="226" spans="1:4" x14ac:dyDescent="0.25">
@@ -5369,10 +5368,10 @@
         <v>447</v>
       </c>
       <c r="C226" s="4">
-        <v>0.7</v>
+        <v>0.3</v>
       </c>
       <c r="D226" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="227" spans="1:4" x14ac:dyDescent="0.25">
@@ -5383,10 +5382,10 @@
         <v>449</v>
       </c>
       <c r="C227" s="4">
-        <v>0.7</v>
+        <v>0.3</v>
       </c>
       <c r="D227" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="228" spans="1:4" x14ac:dyDescent="0.25">
@@ -5397,10 +5396,10 @@
         <v>451</v>
       </c>
       <c r="C228" s="4">
-        <v>0.7</v>
+        <v>0.3</v>
       </c>
       <c r="D228" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="229" spans="1:4" x14ac:dyDescent="0.25">
@@ -5411,10 +5410,10 @@
         <v>453</v>
       </c>
       <c r="C229" s="4">
-        <v>0.7</v>
+        <v>0.3</v>
       </c>
       <c r="D229" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="230" spans="1:4" x14ac:dyDescent="0.25">
@@ -5425,10 +5424,10 @@
         <v>455</v>
       </c>
       <c r="C230" s="4">
-        <v>0.7</v>
+        <v>0.3</v>
       </c>
       <c r="D230" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="231" spans="1:4" x14ac:dyDescent="0.25">
@@ -5439,10 +5438,10 @@
         <v>457</v>
       </c>
       <c r="C231" s="4">
-        <v>0.7</v>
+        <v>0.3</v>
       </c>
       <c r="D231" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="232" spans="1:4" x14ac:dyDescent="0.25">
@@ -5453,10 +5452,10 @@
         <v>459</v>
       </c>
       <c r="C232" s="4">
-        <v>0.7</v>
+        <v>0.3</v>
       </c>
       <c r="D232" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="233" spans="1:4" x14ac:dyDescent="0.25">
@@ -5467,10 +5466,10 @@
         <v>461</v>
       </c>
       <c r="C233" s="4">
-        <v>0.7</v>
+        <v>0.3</v>
       </c>
       <c r="D233" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="234" spans="1:4" x14ac:dyDescent="0.25">
@@ -5481,10 +5480,10 @@
         <v>463</v>
       </c>
       <c r="C234" s="4">
-        <v>0.7</v>
+        <v>0.3</v>
       </c>
       <c r="D234" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="235" spans="1:4" x14ac:dyDescent="0.25">
@@ -5495,10 +5494,10 @@
         <v>465</v>
       </c>
       <c r="C235" s="4">
-        <v>0.7</v>
+        <v>0.3</v>
       </c>
       <c r="D235" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="236" spans="1:4" x14ac:dyDescent="0.25">
@@ -5509,10 +5508,10 @@
         <v>467</v>
       </c>
       <c r="C236" s="4">
-        <v>0.7</v>
+        <v>0.3</v>
       </c>
       <c r="D236" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="237" spans="1:4" x14ac:dyDescent="0.25">
@@ -5523,10 +5522,10 @@
         <v>469</v>
       </c>
       <c r="C237" s="4">
-        <v>0.7</v>
+        <v>0.3</v>
       </c>
       <c r="D237" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="238" spans="1:4" x14ac:dyDescent="0.25">
@@ -5537,10 +5536,10 @@
         <v>471</v>
       </c>
       <c r="C238" s="4">
-        <v>0.7</v>
+        <v>0.3</v>
       </c>
       <c r="D238" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="239" spans="1:4" x14ac:dyDescent="0.25">
@@ -5551,10 +5550,10 @@
         <v>473</v>
       </c>
       <c r="C239" s="4">
-        <v>0.7</v>
+        <v>0.3</v>
       </c>
       <c r="D239" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="240" spans="1:4" x14ac:dyDescent="0.25">
@@ -5565,10 +5564,10 @@
         <v>475</v>
       </c>
       <c r="C240" s="4">
-        <v>0.7</v>
+        <v>0.3</v>
       </c>
       <c r="D240" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="241" spans="1:4" x14ac:dyDescent="0.25">
@@ -5579,10 +5578,10 @@
         <v>477</v>
       </c>
       <c r="C241" s="4">
-        <v>0.7</v>
+        <v>0.3</v>
       </c>
       <c r="D241" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="242" spans="1:4" x14ac:dyDescent="0.25">
@@ -5593,10 +5592,10 @@
         <v>479</v>
       </c>
       <c r="C242" s="4">
-        <v>0.7</v>
+        <v>0.3</v>
       </c>
       <c r="D242" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="243" spans="1:4" x14ac:dyDescent="0.25">
@@ -5607,10 +5606,10 @@
         <v>481</v>
       </c>
       <c r="C243" s="4">
-        <v>0.7</v>
+        <v>0.3</v>
       </c>
       <c r="D243" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="244" spans="1:4" x14ac:dyDescent="0.25">
@@ -5621,10 +5620,10 @@
         <v>483</v>
       </c>
       <c r="C244" s="4">
-        <v>0.7</v>
+        <v>0.3</v>
       </c>
       <c r="D244" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="245" spans="1:4" x14ac:dyDescent="0.25">
@@ -5635,10 +5634,10 @@
         <v>485</v>
       </c>
       <c r="C245" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D245" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="246" spans="1:4" x14ac:dyDescent="0.25">
@@ -5649,10 +5648,10 @@
         <v>487</v>
       </c>
       <c r="C246" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D246" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="247" spans="1:4" x14ac:dyDescent="0.25">
@@ -5663,10 +5662,10 @@
         <v>489</v>
       </c>
       <c r="C247" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D247" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="248" spans="1:4" x14ac:dyDescent="0.25">
@@ -5677,10 +5676,10 @@
         <v>491</v>
       </c>
       <c r="C248" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D248" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="249" spans="1:4" x14ac:dyDescent="0.25">
@@ -5691,10 +5690,10 @@
         <v>493</v>
       </c>
       <c r="C249" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D249" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="250" spans="1:4" x14ac:dyDescent="0.25">
@@ -5705,10 +5704,10 @@
         <v>495</v>
       </c>
       <c r="C250" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D250" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="251" spans="1:4" x14ac:dyDescent="0.25">
@@ -5719,10 +5718,10 @@
         <v>497</v>
       </c>
       <c r="C251" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D251" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="252" spans="1:4" x14ac:dyDescent="0.25">
@@ -5733,10 +5732,10 @@
         <v>499</v>
       </c>
       <c r="C252" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D252" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="253" spans="1:4" x14ac:dyDescent="0.25">
@@ -5747,10 +5746,10 @@
         <v>501</v>
       </c>
       <c r="C253" s="4">
-        <v>0.7</v>
+        <v>0.2</v>
       </c>
       <c r="D253" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="254" spans="1:4" x14ac:dyDescent="0.25">
@@ -5761,10 +5760,10 @@
         <v>503</v>
       </c>
       <c r="C254" s="4">
-        <v>0.7</v>
+        <v>0.2</v>
       </c>
       <c r="D254" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="255" spans="1:4" x14ac:dyDescent="0.25">
@@ -5775,10 +5774,10 @@
         <v>505</v>
       </c>
       <c r="C255" s="4">
-        <v>0.7</v>
+        <v>0.2</v>
       </c>
       <c r="D255" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="256" spans="1:4" x14ac:dyDescent="0.25">
@@ -5789,10 +5788,10 @@
         <v>507</v>
       </c>
       <c r="C256" s="4">
-        <v>0.7</v>
+        <v>0.2</v>
       </c>
       <c r="D256" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="257" spans="1:4" x14ac:dyDescent="0.25">
@@ -5803,10 +5802,10 @@
         <v>509</v>
       </c>
       <c r="C257" s="4">
-        <v>0.7</v>
+        <v>0.2</v>
       </c>
       <c r="D257" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="258" spans="1:4" x14ac:dyDescent="0.25">
@@ -5817,10 +5816,10 @@
         <v>511</v>
       </c>
       <c r="C258" s="4">
-        <v>0.7</v>
+        <v>0.2</v>
       </c>
       <c r="D258" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="259" spans="1:4" x14ac:dyDescent="0.25">
@@ -5831,10 +5830,10 @@
         <v>513</v>
       </c>
       <c r="C259" s="4">
-        <v>0.7</v>
+        <v>0.2</v>
       </c>
       <c r="D259" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="260" spans="1:4" x14ac:dyDescent="0.25">
@@ -5845,10 +5844,10 @@
         <v>515</v>
       </c>
       <c r="C260" s="4">
-        <v>0.7</v>
+        <v>0.2</v>
       </c>
       <c r="D260" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="261" spans="1:4" x14ac:dyDescent="0.25">
@@ -5859,10 +5858,10 @@
         <v>517</v>
       </c>
       <c r="C261" s="4">
-        <v>0.7</v>
+        <v>0.2</v>
       </c>
       <c r="D261" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="262" spans="1:4" x14ac:dyDescent="0.25">
@@ -5873,10 +5872,10 @@
         <v>519</v>
       </c>
       <c r="C262" s="4">
-        <v>0.7</v>
+        <v>0.2</v>
       </c>
       <c r="D262" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="263" spans="1:4" x14ac:dyDescent="0.25">
@@ -5887,10 +5886,10 @@
         <v>521</v>
       </c>
       <c r="C263" s="4">
-        <v>0.7</v>
+        <v>0.2</v>
       </c>
       <c r="D263" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="264" spans="1:4" x14ac:dyDescent="0.25">
@@ -5901,10 +5900,10 @@
         <v>523</v>
       </c>
       <c r="C264" s="4">
-        <v>0.7</v>
+        <v>0.2</v>
       </c>
       <c r="D264" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="265" spans="1:4" x14ac:dyDescent="0.25">
@@ -5915,10 +5914,10 @@
         <v>525</v>
       </c>
       <c r="C265" s="4">
-        <v>0.7</v>
+        <v>0.2</v>
       </c>
       <c r="D265" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="266" spans="1:4" x14ac:dyDescent="0.25">
@@ -5929,10 +5928,10 @@
         <v>527</v>
       </c>
       <c r="C266" s="4">
-        <v>0.7</v>
+        <v>0.2</v>
       </c>
       <c r="D266" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="267" spans="1:4" x14ac:dyDescent="0.25">
@@ -5943,10 +5942,10 @@
         <v>529</v>
       </c>
       <c r="C267" s="4">
-        <v>0.7</v>
+        <v>0.2</v>
       </c>
       <c r="D267" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="268" spans="1:4" x14ac:dyDescent="0.25">
@@ -5957,10 +5956,10 @@
         <v>531</v>
       </c>
       <c r="C268" s="4">
-        <v>0.7</v>
+        <v>0.2</v>
       </c>
       <c r="D268" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="269" spans="1:4" x14ac:dyDescent="0.25">
@@ -5971,10 +5970,10 @@
         <v>533</v>
       </c>
       <c r="C269" s="4">
-        <v>0.7</v>
+        <v>0.2</v>
       </c>
       <c r="D269" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="270" spans="1:4" x14ac:dyDescent="0.25">
@@ -5985,10 +5984,10 @@
         <v>535</v>
       </c>
       <c r="C270" s="4">
-        <v>0.7</v>
+        <v>0.2</v>
       </c>
       <c r="D270" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="271" spans="1:4" x14ac:dyDescent="0.25">
@@ -5999,10 +5998,10 @@
         <v>537</v>
       </c>
       <c r="C271" s="4">
-        <v>0.7</v>
+        <v>0.2</v>
       </c>
       <c r="D271" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="272" spans="1:4" x14ac:dyDescent="0.25">
@@ -6013,10 +6012,10 @@
         <v>539</v>
       </c>
       <c r="C272" s="4">
-        <v>0.7</v>
+        <v>0.2</v>
       </c>
       <c r="D272" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="273" spans="1:4" x14ac:dyDescent="0.25">
@@ -6027,10 +6026,10 @@
         <v>541</v>
       </c>
       <c r="C273" s="4">
-        <v>0.7</v>
+        <v>0.2</v>
       </c>
       <c r="D273" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="274" spans="1:4" x14ac:dyDescent="0.25">
@@ -6041,10 +6040,10 @@
         <v>543</v>
       </c>
       <c r="C274" s="4">
-        <v>0.7</v>
+        <v>0.2</v>
       </c>
       <c r="D274" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="275" spans="1:4" x14ac:dyDescent="0.25">
@@ -6055,10 +6054,10 @@
         <v>545</v>
       </c>
       <c r="C275" s="4">
-        <v>0.7</v>
+        <v>0.2</v>
       </c>
       <c r="D275" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="276" spans="1:4" x14ac:dyDescent="0.25">
@@ -6069,10 +6068,10 @@
         <v>547</v>
       </c>
       <c r="C276" s="4">
-        <v>0.7</v>
+        <v>0.2</v>
       </c>
       <c r="D276" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="277" spans="1:4" x14ac:dyDescent="0.25">
@@ -6083,10 +6082,10 @@
         <v>549</v>
       </c>
       <c r="C277" s="4">
-        <v>0.7</v>
+        <v>0.2</v>
       </c>
       <c r="D277" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="278" spans="1:4" x14ac:dyDescent="0.25">
@@ -6097,10 +6096,10 @@
         <v>551</v>
       </c>
       <c r="C278" s="4">
-        <v>0.7</v>
+        <v>0.2</v>
       </c>
       <c r="D278" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="279" spans="1:4" x14ac:dyDescent="0.25">
@@ -6111,10 +6110,10 @@
         <v>553</v>
       </c>
       <c r="C279" s="4">
-        <v>0.7</v>
+        <v>0.2</v>
       </c>
       <c r="D279" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="280" spans="1:4" x14ac:dyDescent="0.25">
@@ -6125,10 +6124,10 @@
         <v>555</v>
       </c>
       <c r="C280" s="4">
-        <v>0.7</v>
+        <v>0.2</v>
       </c>
       <c r="D280" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="281" spans="1:4" x14ac:dyDescent="0.25">
@@ -6139,10 +6138,10 @@
         <v>557</v>
       </c>
       <c r="C281" s="4">
-        <v>0.7</v>
+        <v>0.2</v>
       </c>
       <c r="D281" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="282" spans="1:4" x14ac:dyDescent="0.25">
@@ -6153,10 +6152,10 @@
         <v>559</v>
       </c>
       <c r="C282" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D282" s="5">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="283" spans="1:4" x14ac:dyDescent="0.25">
@@ -6167,10 +6166,10 @@
         <v>561</v>
       </c>
       <c r="C283" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D283" s="5">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="284" spans="1:4" x14ac:dyDescent="0.25">
@@ -6181,10 +6180,10 @@
         <v>563</v>
       </c>
       <c r="C284" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D284" s="5">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="285" spans="1:4" x14ac:dyDescent="0.25">
@@ -6195,10 +6194,10 @@
         <v>565</v>
       </c>
       <c r="C285" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D285" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="286" spans="1:4" x14ac:dyDescent="0.25">
@@ -6209,10 +6208,10 @@
         <v>567</v>
       </c>
       <c r="C286" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D286" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="287" spans="1:4" x14ac:dyDescent="0.25">
@@ -6223,10 +6222,10 @@
         <v>569</v>
       </c>
       <c r="C287" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D287" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="288" spans="1:4" x14ac:dyDescent="0.25">
@@ -6237,10 +6236,10 @@
         <v>571</v>
       </c>
       <c r="C288" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D288" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="289" spans="1:4" x14ac:dyDescent="0.25">
@@ -6251,10 +6250,10 @@
         <v>573</v>
       </c>
       <c r="C289" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D289" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="290" spans="1:4" x14ac:dyDescent="0.25">
@@ -6265,10 +6264,10 @@
         <v>575</v>
       </c>
       <c r="C290" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D290" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="291" spans="1:4" x14ac:dyDescent="0.25">
@@ -6279,7 +6278,7 @@
         <v>577</v>
       </c>
       <c r="C291" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D291" s="5">
         <v>0</v>
@@ -6293,7 +6292,7 @@
         <v>579</v>
       </c>
       <c r="C292" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D292" s="5">
         <v>0</v>
@@ -6307,7 +6306,7 @@
         <v>581</v>
       </c>
       <c r="C293" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D293" s="5">
         <v>0</v>
@@ -6321,7 +6320,7 @@
         <v>583</v>
       </c>
       <c r="C294" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D294" s="5">
         <v>0</v>
@@ -6335,7 +6334,7 @@
         <v>585</v>
       </c>
       <c r="C295" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D295" s="5">
         <v>0</v>
@@ -6349,7 +6348,7 @@
         <v>587</v>
       </c>
       <c r="C296" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D296" s="5">
         <v>0</v>
@@ -6363,7 +6362,7 @@
         <v>589</v>
       </c>
       <c r="C297" s="4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="D297" s="5">
         <v>0</v>
@@ -6380,7 +6379,7 @@
         <v>0.7</v>
       </c>
       <c r="D298" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="299" spans="1:4" x14ac:dyDescent="0.25">
@@ -6394,7 +6393,7 @@
         <v>0.7</v>
       </c>
       <c r="D299" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="300" spans="1:4" x14ac:dyDescent="0.25">
@@ -6408,7 +6407,7 @@
         <v>0.7</v>
       </c>
       <c r="D300" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="301" spans="1:4" x14ac:dyDescent="0.25">
@@ -6418,12 +6417,8 @@
       <c r="B301" t="s">
         <v>597</v>
       </c>
-      <c r="C301" s="4">
-        <v>0.7</v>
-      </c>
-      <c r="D301" s="5">
-        <v>0</v>
-      </c>
+      <c r="C301" s="4"/>
+      <c r="D301" s="5"/>
     </row>
     <row r="302" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A302" t="s">
@@ -6432,12 +6427,8 @@
       <c r="B302" t="s">
         <v>599</v>
       </c>
-      <c r="C302" s="4">
-        <v>0.7</v>
-      </c>
-      <c r="D302" s="5">
-        <v>0</v>
-      </c>
+      <c r="C302" s="4"/>
+      <c r="D302" s="5"/>
     </row>
     <row r="303" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A303" t="s">
@@ -6447,10 +6438,11 @@
         <v>601</v>
       </c>
       <c r="C303" s="4">
-        <v>0.7</v>
+        <f>1/3</f>
+        <v>0.33333333333333331</v>
       </c>
       <c r="D303" s="5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix allocation defaults, category labels, and default allocation loading in app_2021
</commit_message>
<xml_diff>
--- a/Allocation Input Form.xlsx
+++ b/Allocation Input Form.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29713"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mszekely\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mszek\OneDrive\Desktop\2019SHS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C6D9FEED-3418-4D94-BBE9-D9ACE0A64CE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{332CB63C-07C6-4504-98C1-789DD4527DF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2490" yWindow="0" windowWidth="25170" windowHeight="21705" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-12615" yWindow="-21720" windowWidth="51840" windowHeight="21840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Spending Estimates" sheetId="1" r:id="rId1"/>
@@ -2230,8 +2230,7 @@
   <dimension ref="A1:D303"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="50" customWidth="1"/>
-    <col min="2" max="2" width="59.42578125" customWidth="1"/>
+    <col min="1" max="2" width="50" customWidth="1"/>
     <col min="3" max="3" width="26.5703125" style="1" customWidth="1"/>
     <col min="4" max="4" width="23.28515625" style="1" customWidth="1"/>
   </cols>
@@ -2276,9 +2275,11 @@
         <v>6</v>
       </c>
       <c r="C5" s="4">
-        <v>0</v>
-      </c>
-      <c r="D5" s="5"/>
+        <v>0.7</v>
+      </c>
+      <c r="D5" s="5">
+        <v>4</v>
+      </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
@@ -2288,7 +2289,7 @@
         <v>8</v>
       </c>
       <c r="C6" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D6" s="5">
         <v>4</v>
@@ -2302,10 +2303,10 @@
         <v>10</v>
       </c>
       <c r="C7" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D7" s="5">
-        <v>4.0011997600479905</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -2316,7 +2317,7 @@
         <v>12</v>
       </c>
       <c r="C8" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D8" s="5">
         <v>4</v>
@@ -2330,7 +2331,7 @@
         <v>14</v>
       </c>
       <c r="C9" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D9" s="5">
         <v>4</v>
@@ -2344,7 +2345,7 @@
         <v>16</v>
       </c>
       <c r="C10" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D10" s="5">
         <v>4</v>
@@ -2358,7 +2359,7 @@
         <v>18</v>
       </c>
       <c r="C11" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D11" s="5">
         <v>4</v>
@@ -2372,7 +2373,7 @@
         <v>20</v>
       </c>
       <c r="C12" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D12" s="5">
         <v>4</v>
@@ -2386,7 +2387,7 @@
         <v>22</v>
       </c>
       <c r="C13" s="4">
-        <v>0</v>
+        <v>0.65</v>
       </c>
       <c r="D13" s="5">
         <v>4</v>
@@ -2400,7 +2401,7 @@
         <v>24</v>
       </c>
       <c r="C14" s="4">
-        <v>0</v>
+        <v>0.65</v>
       </c>
       <c r="D14" s="5">
         <v>4</v>
@@ -2414,7 +2415,7 @@
         <v>26</v>
       </c>
       <c r="C15" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D15" s="5">
         <v>4</v>
@@ -2428,7 +2429,7 @@
         <v>28</v>
       </c>
       <c r="C16" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D16" s="5">
         <v>4</v>
@@ -2442,7 +2443,7 @@
         <v>30</v>
       </c>
       <c r="C17" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D17" s="5">
         <v>4</v>
@@ -2456,7 +2457,7 @@
         <v>32</v>
       </c>
       <c r="C18" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D18" s="5">
         <v>4</v>
@@ -2470,7 +2471,7 @@
         <v>34</v>
       </c>
       <c r="C19" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D19" s="5">
         <v>4</v>
@@ -2484,7 +2485,7 @@
         <v>36</v>
       </c>
       <c r="C20" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D20" s="5">
         <v>4</v>
@@ -2498,7 +2499,7 @@
         <v>38</v>
       </c>
       <c r="C21" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D21" s="5">
         <v>4</v>
@@ -2512,7 +2513,7 @@
         <v>40</v>
       </c>
       <c r="C22" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D22" s="5">
         <v>4</v>
@@ -2526,7 +2527,7 @@
         <v>42</v>
       </c>
       <c r="C23" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D23" s="5">
         <v>4</v>
@@ -2540,7 +2541,7 @@
         <v>44</v>
       </c>
       <c r="C24" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D24" s="5">
         <v>4</v>
@@ -2554,7 +2555,7 @@
         <v>46</v>
       </c>
       <c r="C25" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D25" s="5">
         <v>4</v>
@@ -2568,7 +2569,7 @@
         <v>48</v>
       </c>
       <c r="C26" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D26" s="5">
         <v>4</v>
@@ -2582,7 +2583,7 @@
         <v>50</v>
       </c>
       <c r="C27" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D27" s="5">
         <v>4</v>
@@ -2596,7 +2597,7 @@
         <v>52</v>
       </c>
       <c r="C28" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D28" s="5">
         <v>4</v>
@@ -2610,7 +2611,7 @@
         <v>54</v>
       </c>
       <c r="C29" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D29" s="5">
         <v>4</v>
@@ -2624,7 +2625,7 @@
         <v>56</v>
       </c>
       <c r="C30" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D30" s="5">
         <v>4</v>
@@ -2638,7 +2639,7 @@
         <v>58</v>
       </c>
       <c r="C31" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D31" s="5">
         <v>4</v>
@@ -2652,7 +2653,7 @@
         <v>60</v>
       </c>
       <c r="C32" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D32" s="5">
         <v>4</v>
@@ -2666,7 +2667,7 @@
         <v>62</v>
       </c>
       <c r="C33" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D33" s="5">
         <v>4</v>
@@ -2680,7 +2681,7 @@
         <v>64</v>
       </c>
       <c r="C34" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D34" s="5">
         <v>4</v>
@@ -2694,7 +2695,7 @@
         <v>66</v>
       </c>
       <c r="C35" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D35" s="5">
         <v>4</v>
@@ -2708,7 +2709,7 @@
         <v>68</v>
       </c>
       <c r="C36" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D36" s="5">
         <v>4</v>
@@ -2722,7 +2723,7 @@
         <v>70</v>
       </c>
       <c r="C37" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D37" s="5">
         <v>4</v>
@@ -2736,7 +2737,7 @@
         <v>72</v>
       </c>
       <c r="C38" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D38" s="5">
         <v>4</v>
@@ -2750,7 +2751,7 @@
         <v>74</v>
       </c>
       <c r="C39" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D39" s="5">
         <v>4</v>
@@ -2764,7 +2765,7 @@
         <v>76</v>
       </c>
       <c r="C40" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D40" s="5">
         <v>4</v>
@@ -2778,7 +2779,7 @@
         <v>78</v>
       </c>
       <c r="C41" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D41" s="5">
         <v>4</v>
@@ -2792,7 +2793,7 @@
         <v>80</v>
       </c>
       <c r="C42" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D42" s="5">
         <v>4</v>
@@ -2806,7 +2807,7 @@
         <v>82</v>
       </c>
       <c r="C43" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D43" s="5">
         <v>4</v>
@@ -2820,7 +2821,7 @@
         <v>84</v>
       </c>
       <c r="C44" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D44" s="5">
         <v>4</v>
@@ -2834,7 +2835,7 @@
         <v>86</v>
       </c>
       <c r="C45" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D45" s="5">
         <v>4</v>
@@ -2848,7 +2849,7 @@
         <v>88</v>
       </c>
       <c r="C46" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D46" s="5">
         <v>4</v>
@@ -2862,7 +2863,7 @@
         <v>90</v>
       </c>
       <c r="C47" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D47" s="5">
         <v>4</v>
@@ -2876,7 +2877,7 @@
         <v>92</v>
       </c>
       <c r="C48" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D48" s="5">
         <v>4</v>
@@ -2890,7 +2891,7 @@
         <v>94</v>
       </c>
       <c r="C49" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D49" s="5">
         <v>4</v>
@@ -2904,7 +2905,7 @@
         <v>96</v>
       </c>
       <c r="C50" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D50" s="5">
         <v>4</v>
@@ -2918,7 +2919,7 @@
         <v>98</v>
       </c>
       <c r="C51" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D51" s="5">
         <v>4</v>
@@ -2932,7 +2933,7 @@
         <v>100</v>
       </c>
       <c r="C52" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D52" s="5">
         <v>4</v>
@@ -2946,7 +2947,7 @@
         <v>102</v>
       </c>
       <c r="C53" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D53" s="5">
         <v>4</v>
@@ -2960,7 +2961,7 @@
         <v>104</v>
       </c>
       <c r="C54" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D54" s="5">
         <v>4</v>
@@ -2974,10 +2975,10 @@
         <v>106</v>
       </c>
       <c r="C55" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D55" s="5">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
@@ -2988,10 +2989,10 @@
         <v>108</v>
       </c>
       <c r="C56" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D56" s="5">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
@@ -3002,10 +3003,10 @@
         <v>110</v>
       </c>
       <c r="C57" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D57" s="5">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
@@ -3016,10 +3017,10 @@
         <v>112</v>
       </c>
       <c r="C58" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D58" s="5">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
@@ -3030,10 +3031,10 @@
         <v>114</v>
       </c>
       <c r="C59" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D59" s="5">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
@@ -3044,10 +3045,10 @@
         <v>116</v>
       </c>
       <c r="C60" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D60" s="5">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
@@ -3058,10 +3059,10 @@
         <v>118</v>
       </c>
       <c r="C61" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D61" s="5">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
@@ -3072,10 +3073,10 @@
         <v>120</v>
       </c>
       <c r="C62" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D62" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
@@ -3086,10 +3087,10 @@
         <v>122</v>
       </c>
       <c r="C63" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D63" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
@@ -3100,10 +3101,10 @@
         <v>124</v>
       </c>
       <c r="C64" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D64" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
@@ -3114,10 +3115,10 @@
         <v>126</v>
       </c>
       <c r="C65" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D65" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
@@ -3128,10 +3129,10 @@
         <v>128</v>
       </c>
       <c r="C66" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D66" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
@@ -3142,10 +3143,10 @@
         <v>130</v>
       </c>
       <c r="C67" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D67" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
@@ -3156,10 +3157,10 @@
         <v>132</v>
       </c>
       <c r="C68" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D68" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
@@ -3170,10 +3171,10 @@
         <v>134</v>
       </c>
       <c r="C69" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D69" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
@@ -3184,10 +3185,10 @@
         <v>136</v>
       </c>
       <c r="C70" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D70" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
@@ -3198,10 +3199,10 @@
         <v>138</v>
       </c>
       <c r="C71" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D71" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
@@ -3212,10 +3213,10 @@
         <v>140</v>
       </c>
       <c r="C72" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D72" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
@@ -3226,10 +3227,10 @@
         <v>142</v>
       </c>
       <c r="C73" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D73" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
@@ -3240,10 +3241,10 @@
         <v>144</v>
       </c>
       <c r="C74" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D74" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
@@ -3254,10 +3255,10 @@
         <v>146</v>
       </c>
       <c r="C75" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D75" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
@@ -3268,10 +3269,10 @@
         <v>148</v>
       </c>
       <c r="C76" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D76" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
@@ -3282,10 +3283,10 @@
         <v>150</v>
       </c>
       <c r="C77" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D77" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
@@ -3296,10 +3297,10 @@
         <v>152</v>
       </c>
       <c r="C78" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D78" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
@@ -3310,10 +3311,10 @@
         <v>154</v>
       </c>
       <c r="C79" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D79" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">
@@ -3324,10 +3325,10 @@
         <v>156</v>
       </c>
       <c r="C80" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D80" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
@@ -3338,10 +3339,10 @@
         <v>158</v>
       </c>
       <c r="C81" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D81" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
@@ -3352,10 +3353,10 @@
         <v>160</v>
       </c>
       <c r="C82" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D82" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
@@ -3366,10 +3367,10 @@
         <v>162</v>
       </c>
       <c r="C83" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D83" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
@@ -3380,10 +3381,10 @@
         <v>164</v>
       </c>
       <c r="C84" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D84" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
@@ -3394,10 +3395,10 @@
         <v>166</v>
       </c>
       <c r="C85" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D85" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
@@ -3408,10 +3409,10 @@
         <v>168</v>
       </c>
       <c r="C86" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D86" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
@@ -3422,10 +3423,10 @@
         <v>170</v>
       </c>
       <c r="C87" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D87" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
@@ -3436,10 +3437,10 @@
         <v>172</v>
       </c>
       <c r="C88" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D88" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
@@ -3450,10 +3451,10 @@
         <v>174</v>
       </c>
       <c r="C89" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D89" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.25">
@@ -3464,10 +3465,10 @@
         <v>176</v>
       </c>
       <c r="C90" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D90" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
@@ -3478,10 +3479,10 @@
         <v>178</v>
       </c>
       <c r="C91" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D91" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.25">
@@ -3492,10 +3493,10 @@
         <v>180</v>
       </c>
       <c r="C92" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D92" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.25">
@@ -3506,10 +3507,10 @@
         <v>182</v>
       </c>
       <c r="C93" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D93" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.25">
@@ -3520,10 +3521,10 @@
         <v>184</v>
       </c>
       <c r="C94" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D94" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.25">
@@ -3534,10 +3535,10 @@
         <v>186</v>
       </c>
       <c r="C95" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D95" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.25">
@@ -3548,10 +3549,10 @@
         <v>188</v>
       </c>
       <c r="C96" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D96" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
@@ -3562,10 +3563,10 @@
         <v>190</v>
       </c>
       <c r="C97" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D97" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
@@ -3576,10 +3577,10 @@
         <v>192</v>
       </c>
       <c r="C98" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D98" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.25">
@@ -3590,10 +3591,10 @@
         <v>194</v>
       </c>
       <c r="C99" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D99" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.25">
@@ -3604,10 +3605,10 @@
         <v>196</v>
       </c>
       <c r="C100" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D100" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.25">
@@ -3618,10 +3619,10 @@
         <v>198</v>
       </c>
       <c r="C101" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D101" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.25">
@@ -3632,10 +3633,10 @@
         <v>200</v>
       </c>
       <c r="C102" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D102" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.25">
@@ -3646,10 +3647,10 @@
         <v>202</v>
       </c>
       <c r="C103" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D103" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.25">
@@ -3660,10 +3661,10 @@
         <v>204</v>
       </c>
       <c r="C104" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D104" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.25">
@@ -3674,10 +3675,10 @@
         <v>206</v>
       </c>
       <c r="C105" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D105" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.25">
@@ -3688,10 +3689,10 @@
         <v>208</v>
       </c>
       <c r="C106" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D106" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.25">
@@ -3702,10 +3703,10 @@
         <v>210</v>
       </c>
       <c r="C107" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D107" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.25">
@@ -3716,10 +3717,10 @@
         <v>212</v>
       </c>
       <c r="C108" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D108" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.25">
@@ -3730,10 +3731,10 @@
         <v>214</v>
       </c>
       <c r="C109" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D109" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.25">
@@ -3744,10 +3745,10 @@
         <v>216</v>
       </c>
       <c r="C110" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D110" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.25">
@@ -3758,10 +3759,10 @@
         <v>218</v>
       </c>
       <c r="C111" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D111" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.25">
@@ -3772,10 +3773,10 @@
         <v>220</v>
       </c>
       <c r="C112" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D112" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.25">
@@ -3786,10 +3787,10 @@
         <v>222</v>
       </c>
       <c r="C113" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D113" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.25">
@@ -3800,10 +3801,10 @@
         <v>224</v>
       </c>
       <c r="C114" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D114" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.25">
@@ -3814,10 +3815,10 @@
         <v>226</v>
       </c>
       <c r="C115" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D115" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.25">
@@ -3828,10 +3829,10 @@
         <v>228</v>
       </c>
       <c r="C116" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D116" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.25">
@@ -3842,10 +3843,10 @@
         <v>230</v>
       </c>
       <c r="C117" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D117" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.25">
@@ -3856,10 +3857,10 @@
         <v>232</v>
       </c>
       <c r="C118" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D118" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.25">
@@ -3870,10 +3871,10 @@
         <v>234</v>
       </c>
       <c r="C119" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D119" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.25">
@@ -3884,10 +3885,10 @@
         <v>236</v>
       </c>
       <c r="C120" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D120" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.25">
@@ -3898,10 +3899,10 @@
         <v>238</v>
       </c>
       <c r="C121" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D121" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.25">
@@ -3912,10 +3913,10 @@
         <v>240</v>
       </c>
       <c r="C122" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D122" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.25">
@@ -3926,10 +3927,10 @@
         <v>242</v>
       </c>
       <c r="C123" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D123" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.25">
@@ -3940,10 +3941,10 @@
         <v>244</v>
       </c>
       <c r="C124" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D124" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="125" spans="1:4" x14ac:dyDescent="0.25">
@@ -3954,10 +3955,10 @@
         <v>246</v>
       </c>
       <c r="C125" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D125" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="126" spans="1:4" x14ac:dyDescent="0.25">
@@ -3968,10 +3969,10 @@
         <v>248</v>
       </c>
       <c r="C126" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D126" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="127" spans="1:4" x14ac:dyDescent="0.25">
@@ -3982,10 +3983,10 @@
         <v>250</v>
       </c>
       <c r="C127" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D127" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="128" spans="1:4" x14ac:dyDescent="0.25">
@@ -3996,10 +3997,10 @@
         <v>252</v>
       </c>
       <c r="C128" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D128" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="129" spans="1:4" x14ac:dyDescent="0.25">
@@ -4010,10 +4011,10 @@
         <v>254</v>
       </c>
       <c r="C129" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D129" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="130" spans="1:4" x14ac:dyDescent="0.25">
@@ -4024,10 +4025,10 @@
         <v>256</v>
       </c>
       <c r="C130" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D130" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="131" spans="1:4" x14ac:dyDescent="0.25">
@@ -4038,10 +4039,10 @@
         <v>258</v>
       </c>
       <c r="C131" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D131" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="132" spans="1:4" x14ac:dyDescent="0.25">
@@ -4052,10 +4053,10 @@
         <v>260</v>
       </c>
       <c r="C132" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D132" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="133" spans="1:4" x14ac:dyDescent="0.25">
@@ -4066,10 +4067,10 @@
         <v>262</v>
       </c>
       <c r="C133" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D133" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="134" spans="1:4" x14ac:dyDescent="0.25">
@@ -4080,10 +4081,10 @@
         <v>264</v>
       </c>
       <c r="C134" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D134" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="135" spans="1:4" x14ac:dyDescent="0.25">
@@ -4094,10 +4095,10 @@
         <v>266</v>
       </c>
       <c r="C135" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D135" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="136" spans="1:4" x14ac:dyDescent="0.25">
@@ -4108,10 +4109,10 @@
         <v>268</v>
       </c>
       <c r="C136" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D136" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="137" spans="1:4" x14ac:dyDescent="0.25">
@@ -4122,10 +4123,10 @@
         <v>270</v>
       </c>
       <c r="C137" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D137" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="138" spans="1:4" x14ac:dyDescent="0.25">
@@ -4136,10 +4137,10 @@
         <v>272</v>
       </c>
       <c r="C138" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D138" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="139" spans="1:4" x14ac:dyDescent="0.25">
@@ -4150,10 +4151,10 @@
         <v>274</v>
       </c>
       <c r="C139" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D139" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="140" spans="1:4" x14ac:dyDescent="0.25">
@@ -4164,10 +4165,10 @@
         <v>276</v>
       </c>
       <c r="C140" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D140" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="141" spans="1:4" x14ac:dyDescent="0.25">
@@ -4178,10 +4179,10 @@
         <v>278</v>
       </c>
       <c r="C141" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D141" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="142" spans="1:4" x14ac:dyDescent="0.25">
@@ -4192,10 +4193,10 @@
         <v>280</v>
       </c>
       <c r="C142" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D142" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="143" spans="1:4" x14ac:dyDescent="0.25">
@@ -4206,10 +4207,10 @@
         <v>282</v>
       </c>
       <c r="C143" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D143" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="144" spans="1:4" x14ac:dyDescent="0.25">
@@ -4220,10 +4221,10 @@
         <v>284</v>
       </c>
       <c r="C144" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D144" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="145" spans="1:4" x14ac:dyDescent="0.25">
@@ -4234,10 +4235,10 @@
         <v>286</v>
       </c>
       <c r="C145" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D145" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="146" spans="1:4" x14ac:dyDescent="0.25">
@@ -4248,10 +4249,10 @@
         <v>288</v>
       </c>
       <c r="C146" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D146" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="147" spans="1:4" x14ac:dyDescent="0.25">
@@ -4262,10 +4263,10 @@
         <v>290</v>
       </c>
       <c r="C147" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D147" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="148" spans="1:4" x14ac:dyDescent="0.25">
@@ -4276,10 +4277,10 @@
         <v>292</v>
       </c>
       <c r="C148" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D148" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="149" spans="1:4" x14ac:dyDescent="0.25">
@@ -4290,10 +4291,10 @@
         <v>294</v>
       </c>
       <c r="C149" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D149" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="150" spans="1:4" x14ac:dyDescent="0.25">
@@ -4304,10 +4305,10 @@
         <v>296</v>
       </c>
       <c r="C150" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D150" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="151" spans="1:4" x14ac:dyDescent="0.25">
@@ -4318,10 +4319,10 @@
         <v>298</v>
       </c>
       <c r="C151" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D151" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="152" spans="1:4" x14ac:dyDescent="0.25">
@@ -4332,10 +4333,10 @@
         <v>300</v>
       </c>
       <c r="C152" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D152" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="153" spans="1:4" x14ac:dyDescent="0.25">
@@ -4346,10 +4347,10 @@
         <v>302</v>
       </c>
       <c r="C153" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D153" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="154" spans="1:4" x14ac:dyDescent="0.25">
@@ -4360,10 +4361,10 @@
         <v>304</v>
       </c>
       <c r="C154" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D154" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="155" spans="1:4" x14ac:dyDescent="0.25">
@@ -4374,10 +4375,10 @@
         <v>306</v>
       </c>
       <c r="C155" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D155" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="156" spans="1:4" x14ac:dyDescent="0.25">
@@ -4388,10 +4389,10 @@
         <v>308</v>
       </c>
       <c r="C156" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D156" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="157" spans="1:4" x14ac:dyDescent="0.25">
@@ -4402,10 +4403,10 @@
         <v>310</v>
       </c>
       <c r="C157" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D157" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="158" spans="1:4" x14ac:dyDescent="0.25">
@@ -4416,10 +4417,10 @@
         <v>312</v>
       </c>
       <c r="C158" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D158" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="159" spans="1:4" x14ac:dyDescent="0.25">
@@ -4430,10 +4431,10 @@
         <v>314</v>
       </c>
       <c r="C159" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D159" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="160" spans="1:4" x14ac:dyDescent="0.25">
@@ -4444,10 +4445,10 @@
         <v>316</v>
       </c>
       <c r="C160" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D160" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="161" spans="1:4" x14ac:dyDescent="0.25">
@@ -4458,10 +4459,10 @@
         <v>318</v>
       </c>
       <c r="C161" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D161" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="162" spans="1:4" x14ac:dyDescent="0.25">
@@ -4472,10 +4473,10 @@
         <v>320</v>
       </c>
       <c r="C162" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D162" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="163" spans="1:4" x14ac:dyDescent="0.25">
@@ -4489,7 +4490,7 @@
         <v>0.7</v>
       </c>
       <c r="D163" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="164" spans="1:4" x14ac:dyDescent="0.25">
@@ -4503,7 +4504,7 @@
         <v>0.7</v>
       </c>
       <c r="D164" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="165" spans="1:4" x14ac:dyDescent="0.25">
@@ -4517,7 +4518,7 @@
         <v>0.7</v>
       </c>
       <c r="D165" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="166" spans="1:4" x14ac:dyDescent="0.25">
@@ -4531,7 +4532,7 @@
         <v>0.7</v>
       </c>
       <c r="D166" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="167" spans="1:4" x14ac:dyDescent="0.25">
@@ -4545,7 +4546,7 @@
         <v>0.7</v>
       </c>
       <c r="D167" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="168" spans="1:4" x14ac:dyDescent="0.25">
@@ -4559,7 +4560,7 @@
         <v>0.7</v>
       </c>
       <c r="D168" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="169" spans="1:4" x14ac:dyDescent="0.25">
@@ -4573,7 +4574,7 @@
         <v>0.7</v>
       </c>
       <c r="D169" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="170" spans="1:4" x14ac:dyDescent="0.25">
@@ -4587,7 +4588,7 @@
         <v>0.7</v>
       </c>
       <c r="D170" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="171" spans="1:4" x14ac:dyDescent="0.25">
@@ -4601,7 +4602,7 @@
         <v>0.7</v>
       </c>
       <c r="D171" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="172" spans="1:4" x14ac:dyDescent="0.25">
@@ -4615,7 +4616,7 @@
         <v>0.7</v>
       </c>
       <c r="D172" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="173" spans="1:4" x14ac:dyDescent="0.25">
@@ -4629,7 +4630,7 @@
         <v>0.7</v>
       </c>
       <c r="D173" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="174" spans="1:4" x14ac:dyDescent="0.25">
@@ -4643,7 +4644,7 @@
         <v>0.7</v>
       </c>
       <c r="D174" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="175" spans="1:4" x14ac:dyDescent="0.25">
@@ -4657,7 +4658,7 @@
         <v>0.7</v>
       </c>
       <c r="D175" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="176" spans="1:4" x14ac:dyDescent="0.25">
@@ -4671,7 +4672,7 @@
         <v>0.7</v>
       </c>
       <c r="D176" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="177" spans="1:4" x14ac:dyDescent="0.25">
@@ -4685,7 +4686,7 @@
         <v>0.7</v>
       </c>
       <c r="D177" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="178" spans="1:4" x14ac:dyDescent="0.25">
@@ -4699,7 +4700,7 @@
         <v>0.7</v>
       </c>
       <c r="D178" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="179" spans="1:4" x14ac:dyDescent="0.25">
@@ -4713,7 +4714,7 @@
         <v>0.7</v>
       </c>
       <c r="D179" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="180" spans="1:4" x14ac:dyDescent="0.25">
@@ -4727,7 +4728,7 @@
         <v>0.7</v>
       </c>
       <c r="D180" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="181" spans="1:4" x14ac:dyDescent="0.25">
@@ -4741,7 +4742,7 @@
         <v>0.7</v>
       </c>
       <c r="D181" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="182" spans="1:4" x14ac:dyDescent="0.25">
@@ -4755,7 +4756,7 @@
         <v>0.7</v>
       </c>
       <c r="D182" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="183" spans="1:4" x14ac:dyDescent="0.25">
@@ -4769,7 +4770,7 @@
         <v>0.7</v>
       </c>
       <c r="D183" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="184" spans="1:4" x14ac:dyDescent="0.25">
@@ -5035,7 +5036,7 @@
         <v>0.7</v>
       </c>
       <c r="D202" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="203" spans="1:4" x14ac:dyDescent="0.25">
@@ -5049,7 +5050,7 @@
         <v>0.7</v>
       </c>
       <c r="D203" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="204" spans="1:4" x14ac:dyDescent="0.25">
@@ -5063,7 +5064,7 @@
         <v>0.7</v>
       </c>
       <c r="D204" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="205" spans="1:4" x14ac:dyDescent="0.25">
@@ -5077,7 +5078,7 @@
         <v>0.7</v>
       </c>
       <c r="D205" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="206" spans="1:4" x14ac:dyDescent="0.25">
@@ -5091,7 +5092,7 @@
         <v>0.7</v>
       </c>
       <c r="D206" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="207" spans="1:4" x14ac:dyDescent="0.25">
@@ -5105,7 +5106,7 @@
         <v>0.7</v>
       </c>
       <c r="D207" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="208" spans="1:4" x14ac:dyDescent="0.25">
@@ -5119,7 +5120,7 @@
         <v>0.7</v>
       </c>
       <c r="D208" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="209" spans="1:4" x14ac:dyDescent="0.25">
@@ -5133,7 +5134,7 @@
         <v>0.7</v>
       </c>
       <c r="D209" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="210" spans="1:4" x14ac:dyDescent="0.25">
@@ -5147,7 +5148,7 @@
         <v>0.7</v>
       </c>
       <c r="D210" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="211" spans="1:4" x14ac:dyDescent="0.25">
@@ -5161,7 +5162,7 @@
         <v>0.7</v>
       </c>
       <c r="D211" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="212" spans="1:4" x14ac:dyDescent="0.25">
@@ -5175,7 +5176,7 @@
         <v>0.7</v>
       </c>
       <c r="D212" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="213" spans="1:4" x14ac:dyDescent="0.25">
@@ -5189,7 +5190,7 @@
         <v>0.7</v>
       </c>
       <c r="D213" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="214" spans="1:4" x14ac:dyDescent="0.25">
@@ -5203,7 +5204,7 @@
         <v>0.7</v>
       </c>
       <c r="D214" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="215" spans="1:4" x14ac:dyDescent="0.25">
@@ -5217,7 +5218,7 @@
         <v>0.7</v>
       </c>
       <c r="D215" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="216" spans="1:4" x14ac:dyDescent="0.25">
@@ -5231,7 +5232,7 @@
         <v>0.7</v>
       </c>
       <c r="D216" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="217" spans="1:4" x14ac:dyDescent="0.25">
@@ -5242,10 +5243,10 @@
         <v>429</v>
       </c>
       <c r="C217" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D217" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="218" spans="1:4" x14ac:dyDescent="0.25">
@@ -5256,10 +5257,10 @@
         <v>431</v>
       </c>
       <c r="C218" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D218" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="219" spans="1:4" x14ac:dyDescent="0.25">
@@ -5270,10 +5271,10 @@
         <v>433</v>
       </c>
       <c r="C219" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D219" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="220" spans="1:4" x14ac:dyDescent="0.25">
@@ -5284,10 +5285,10 @@
         <v>435</v>
       </c>
       <c r="C220" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D220" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="221" spans="1:4" x14ac:dyDescent="0.25">
@@ -5298,10 +5299,10 @@
         <v>437</v>
       </c>
       <c r="C221" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D221" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="222" spans="1:4" x14ac:dyDescent="0.25">
@@ -5312,10 +5313,10 @@
         <v>439</v>
       </c>
       <c r="C222" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D222" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="223" spans="1:4" x14ac:dyDescent="0.25">
@@ -5326,10 +5327,10 @@
         <v>441</v>
       </c>
       <c r="C223" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D223" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="224" spans="1:4" x14ac:dyDescent="0.25">
@@ -5340,10 +5341,10 @@
         <v>443</v>
       </c>
       <c r="C224" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D224" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="225" spans="1:4" x14ac:dyDescent="0.25">
@@ -5354,10 +5355,10 @@
         <v>445</v>
       </c>
       <c r="C225" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D225" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="226" spans="1:4" x14ac:dyDescent="0.25">
@@ -5368,10 +5369,10 @@
         <v>447</v>
       </c>
       <c r="C226" s="4">
-        <v>0.3</v>
+        <v>0.7</v>
       </c>
       <c r="D226" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="227" spans="1:4" x14ac:dyDescent="0.25">
@@ -5382,10 +5383,10 @@
         <v>449</v>
       </c>
       <c r="C227" s="4">
-        <v>0.3</v>
+        <v>0.7</v>
       </c>
       <c r="D227" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="228" spans="1:4" x14ac:dyDescent="0.25">
@@ -5396,10 +5397,10 @@
         <v>451</v>
       </c>
       <c r="C228" s="4">
-        <v>0.3</v>
+        <v>0.7</v>
       </c>
       <c r="D228" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="229" spans="1:4" x14ac:dyDescent="0.25">
@@ -5410,10 +5411,10 @@
         <v>453</v>
       </c>
       <c r="C229" s="4">
-        <v>0.3</v>
+        <v>0.7</v>
       </c>
       <c r="D229" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="230" spans="1:4" x14ac:dyDescent="0.25">
@@ -5424,10 +5425,10 @@
         <v>455</v>
       </c>
       <c r="C230" s="4">
-        <v>0.3</v>
+        <v>0.7</v>
       </c>
       <c r="D230" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="231" spans="1:4" x14ac:dyDescent="0.25">
@@ -5438,10 +5439,10 @@
         <v>457</v>
       </c>
       <c r="C231" s="4">
-        <v>0.3</v>
+        <v>0.7</v>
       </c>
       <c r="D231" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="232" spans="1:4" x14ac:dyDescent="0.25">
@@ -5452,10 +5453,10 @@
         <v>459</v>
       </c>
       <c r="C232" s="4">
-        <v>0.3</v>
+        <v>0.7</v>
       </c>
       <c r="D232" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="233" spans="1:4" x14ac:dyDescent="0.25">
@@ -5466,10 +5467,10 @@
         <v>461</v>
       </c>
       <c r="C233" s="4">
-        <v>0.3</v>
+        <v>0.7</v>
       </c>
       <c r="D233" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="234" spans="1:4" x14ac:dyDescent="0.25">
@@ -5480,10 +5481,10 @@
         <v>463</v>
       </c>
       <c r="C234" s="4">
-        <v>0.3</v>
+        <v>0.7</v>
       </c>
       <c r="D234" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="235" spans="1:4" x14ac:dyDescent="0.25">
@@ -5494,10 +5495,10 @@
         <v>465</v>
       </c>
       <c r="C235" s="4">
-        <v>0.3</v>
+        <v>0.7</v>
       </c>
       <c r="D235" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="236" spans="1:4" x14ac:dyDescent="0.25">
@@ -5508,10 +5509,10 @@
         <v>467</v>
       </c>
       <c r="C236" s="4">
-        <v>0.3</v>
+        <v>0.7</v>
       </c>
       <c r="D236" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="237" spans="1:4" x14ac:dyDescent="0.25">
@@ -5522,10 +5523,10 @@
         <v>469</v>
       </c>
       <c r="C237" s="4">
-        <v>0.3</v>
+        <v>0.7</v>
       </c>
       <c r="D237" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="238" spans="1:4" x14ac:dyDescent="0.25">
@@ -5536,10 +5537,10 @@
         <v>471</v>
       </c>
       <c r="C238" s="4">
-        <v>0.3</v>
+        <v>0.7</v>
       </c>
       <c r="D238" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="239" spans="1:4" x14ac:dyDescent="0.25">
@@ -5550,10 +5551,10 @@
         <v>473</v>
       </c>
       <c r="C239" s="4">
-        <v>0.3</v>
+        <v>0.7</v>
       </c>
       <c r="D239" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="240" spans="1:4" x14ac:dyDescent="0.25">
@@ -5564,10 +5565,10 @@
         <v>475</v>
       </c>
       <c r="C240" s="4">
-        <v>0.3</v>
+        <v>0.7</v>
       </c>
       <c r="D240" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="241" spans="1:4" x14ac:dyDescent="0.25">
@@ -5578,10 +5579,10 @@
         <v>477</v>
       </c>
       <c r="C241" s="4">
-        <v>0.3</v>
+        <v>0.7</v>
       </c>
       <c r="D241" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="242" spans="1:4" x14ac:dyDescent="0.25">
@@ -5592,10 +5593,10 @@
         <v>479</v>
       </c>
       <c r="C242" s="4">
-        <v>0.3</v>
+        <v>0.7</v>
       </c>
       <c r="D242" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="243" spans="1:4" x14ac:dyDescent="0.25">
@@ -5606,10 +5607,10 @@
         <v>481</v>
       </c>
       <c r="C243" s="4">
-        <v>0.3</v>
+        <v>0.7</v>
       </c>
       <c r="D243" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="244" spans="1:4" x14ac:dyDescent="0.25">
@@ -5620,10 +5621,10 @@
         <v>483</v>
       </c>
       <c r="C244" s="4">
-        <v>0.3</v>
+        <v>0.7</v>
       </c>
       <c r="D244" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="245" spans="1:4" x14ac:dyDescent="0.25">
@@ -5634,10 +5635,10 @@
         <v>485</v>
       </c>
       <c r="C245" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D245" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="246" spans="1:4" x14ac:dyDescent="0.25">
@@ -5648,10 +5649,10 @@
         <v>487</v>
       </c>
       <c r="C246" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D246" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="247" spans="1:4" x14ac:dyDescent="0.25">
@@ -5662,10 +5663,10 @@
         <v>489</v>
       </c>
       <c r="C247" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D247" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="248" spans="1:4" x14ac:dyDescent="0.25">
@@ -5676,10 +5677,10 @@
         <v>491</v>
       </c>
       <c r="C248" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D248" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="249" spans="1:4" x14ac:dyDescent="0.25">
@@ -5690,10 +5691,10 @@
         <v>493</v>
       </c>
       <c r="C249" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D249" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="250" spans="1:4" x14ac:dyDescent="0.25">
@@ -5704,10 +5705,10 @@
         <v>495</v>
       </c>
       <c r="C250" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D250" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="251" spans="1:4" x14ac:dyDescent="0.25">
@@ -5718,10 +5719,10 @@
         <v>497</v>
       </c>
       <c r="C251" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D251" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="252" spans="1:4" x14ac:dyDescent="0.25">
@@ -5732,10 +5733,10 @@
         <v>499</v>
       </c>
       <c r="C252" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D252" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="253" spans="1:4" x14ac:dyDescent="0.25">
@@ -5746,10 +5747,10 @@
         <v>501</v>
       </c>
       <c r="C253" s="4">
-        <v>0.2</v>
+        <v>0.7</v>
       </c>
       <c r="D253" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="254" spans="1:4" x14ac:dyDescent="0.25">
@@ -5760,10 +5761,10 @@
         <v>503</v>
       </c>
       <c r="C254" s="4">
-        <v>0.2</v>
+        <v>0.7</v>
       </c>
       <c r="D254" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="255" spans="1:4" x14ac:dyDescent="0.25">
@@ -5774,10 +5775,10 @@
         <v>505</v>
       </c>
       <c r="C255" s="4">
-        <v>0.2</v>
+        <v>0.7</v>
       </c>
       <c r="D255" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="256" spans="1:4" x14ac:dyDescent="0.25">
@@ -5788,10 +5789,10 @@
         <v>507</v>
       </c>
       <c r="C256" s="4">
-        <v>0.2</v>
+        <v>0.7</v>
       </c>
       <c r="D256" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="257" spans="1:4" x14ac:dyDescent="0.25">
@@ -5802,10 +5803,10 @@
         <v>509</v>
       </c>
       <c r="C257" s="4">
-        <v>0.2</v>
+        <v>0.7</v>
       </c>
       <c r="D257" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="258" spans="1:4" x14ac:dyDescent="0.25">
@@ -5816,10 +5817,10 @@
         <v>511</v>
       </c>
       <c r="C258" s="4">
-        <v>0.2</v>
+        <v>0.7</v>
       </c>
       <c r="D258" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="259" spans="1:4" x14ac:dyDescent="0.25">
@@ -5830,10 +5831,10 @@
         <v>513</v>
       </c>
       <c r="C259" s="4">
-        <v>0.2</v>
+        <v>0.7</v>
       </c>
       <c r="D259" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="260" spans="1:4" x14ac:dyDescent="0.25">
@@ -5844,10 +5845,10 @@
         <v>515</v>
       </c>
       <c r="C260" s="4">
-        <v>0.2</v>
+        <v>0.7</v>
       </c>
       <c r="D260" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="261" spans="1:4" x14ac:dyDescent="0.25">
@@ -5858,10 +5859,10 @@
         <v>517</v>
       </c>
       <c r="C261" s="4">
-        <v>0.2</v>
+        <v>0.7</v>
       </c>
       <c r="D261" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="262" spans="1:4" x14ac:dyDescent="0.25">
@@ -5872,10 +5873,10 @@
         <v>519</v>
       </c>
       <c r="C262" s="4">
-        <v>0.2</v>
+        <v>0.7</v>
       </c>
       <c r="D262" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="263" spans="1:4" x14ac:dyDescent="0.25">
@@ -5886,10 +5887,10 @@
         <v>521</v>
       </c>
       <c r="C263" s="4">
-        <v>0.2</v>
+        <v>0.7</v>
       </c>
       <c r="D263" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="264" spans="1:4" x14ac:dyDescent="0.25">
@@ -5900,10 +5901,10 @@
         <v>523</v>
       </c>
       <c r="C264" s="4">
-        <v>0.2</v>
+        <v>0.7</v>
       </c>
       <c r="D264" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="265" spans="1:4" x14ac:dyDescent="0.25">
@@ -5914,10 +5915,10 @@
         <v>525</v>
       </c>
       <c r="C265" s="4">
-        <v>0.2</v>
+        <v>0.7</v>
       </c>
       <c r="D265" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="266" spans="1:4" x14ac:dyDescent="0.25">
@@ -5928,10 +5929,10 @@
         <v>527</v>
       </c>
       <c r="C266" s="4">
-        <v>0.2</v>
+        <v>0.7</v>
       </c>
       <c r="D266" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="267" spans="1:4" x14ac:dyDescent="0.25">
@@ -5942,10 +5943,10 @@
         <v>529</v>
       </c>
       <c r="C267" s="4">
-        <v>0.2</v>
+        <v>0.7</v>
       </c>
       <c r="D267" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="268" spans="1:4" x14ac:dyDescent="0.25">
@@ -5956,10 +5957,10 @@
         <v>531</v>
       </c>
       <c r="C268" s="4">
-        <v>0.2</v>
+        <v>0.7</v>
       </c>
       <c r="D268" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="269" spans="1:4" x14ac:dyDescent="0.25">
@@ -5970,10 +5971,10 @@
         <v>533</v>
       </c>
       <c r="C269" s="4">
-        <v>0.2</v>
+        <v>0.7</v>
       </c>
       <c r="D269" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="270" spans="1:4" x14ac:dyDescent="0.25">
@@ -5984,10 +5985,10 @@
         <v>535</v>
       </c>
       <c r="C270" s="4">
-        <v>0.2</v>
+        <v>0.7</v>
       </c>
       <c r="D270" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="271" spans="1:4" x14ac:dyDescent="0.25">
@@ -5998,10 +5999,10 @@
         <v>537</v>
       </c>
       <c r="C271" s="4">
-        <v>0.2</v>
+        <v>0.7</v>
       </c>
       <c r="D271" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="272" spans="1:4" x14ac:dyDescent="0.25">
@@ -6012,10 +6013,10 @@
         <v>539</v>
       </c>
       <c r="C272" s="4">
-        <v>0.2</v>
+        <v>0.7</v>
       </c>
       <c r="D272" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="273" spans="1:4" x14ac:dyDescent="0.25">
@@ -6026,10 +6027,10 @@
         <v>541</v>
       </c>
       <c r="C273" s="4">
-        <v>0.2</v>
+        <v>0.7</v>
       </c>
       <c r="D273" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="274" spans="1:4" x14ac:dyDescent="0.25">
@@ -6040,10 +6041,10 @@
         <v>543</v>
       </c>
       <c r="C274" s="4">
-        <v>0.2</v>
+        <v>0.7</v>
       </c>
       <c r="D274" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="275" spans="1:4" x14ac:dyDescent="0.25">
@@ -6054,10 +6055,10 @@
         <v>545</v>
       </c>
       <c r="C275" s="4">
-        <v>0.2</v>
+        <v>0.7</v>
       </c>
       <c r="D275" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="276" spans="1:4" x14ac:dyDescent="0.25">
@@ -6068,10 +6069,10 @@
         <v>547</v>
       </c>
       <c r="C276" s="4">
-        <v>0.2</v>
+        <v>0.7</v>
       </c>
       <c r="D276" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="277" spans="1:4" x14ac:dyDescent="0.25">
@@ -6082,10 +6083,10 @@
         <v>549</v>
       </c>
       <c r="C277" s="4">
-        <v>0.2</v>
+        <v>0.7</v>
       </c>
       <c r="D277" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="278" spans="1:4" x14ac:dyDescent="0.25">
@@ -6096,10 +6097,10 @@
         <v>551</v>
       </c>
       <c r="C278" s="4">
-        <v>0.2</v>
+        <v>0.7</v>
       </c>
       <c r="D278" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="279" spans="1:4" x14ac:dyDescent="0.25">
@@ -6110,10 +6111,10 @@
         <v>553</v>
       </c>
       <c r="C279" s="4">
-        <v>0.2</v>
+        <v>0.7</v>
       </c>
       <c r="D279" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="280" spans="1:4" x14ac:dyDescent="0.25">
@@ -6124,10 +6125,10 @@
         <v>555</v>
       </c>
       <c r="C280" s="4">
-        <v>0.2</v>
+        <v>0.7</v>
       </c>
       <c r="D280" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="281" spans="1:4" x14ac:dyDescent="0.25">
@@ -6138,10 +6139,10 @@
         <v>557</v>
       </c>
       <c r="C281" s="4">
-        <v>0.2</v>
+        <v>0.7</v>
       </c>
       <c r="D281" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="282" spans="1:4" x14ac:dyDescent="0.25">
@@ -6152,10 +6153,10 @@
         <v>559</v>
       </c>
       <c r="C282" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D282" s="5">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="283" spans="1:4" x14ac:dyDescent="0.25">
@@ -6166,10 +6167,10 @@
         <v>561</v>
       </c>
       <c r="C283" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D283" s="5">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="284" spans="1:4" x14ac:dyDescent="0.25">
@@ -6180,10 +6181,10 @@
         <v>563</v>
       </c>
       <c r="C284" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D284" s="5">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="285" spans="1:4" x14ac:dyDescent="0.25">
@@ -6194,10 +6195,10 @@
         <v>565</v>
       </c>
       <c r="C285" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D285" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="286" spans="1:4" x14ac:dyDescent="0.25">
@@ -6208,10 +6209,10 @@
         <v>567</v>
       </c>
       <c r="C286" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D286" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="287" spans="1:4" x14ac:dyDescent="0.25">
@@ -6222,10 +6223,10 @@
         <v>569</v>
       </c>
       <c r="C287" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D287" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="288" spans="1:4" x14ac:dyDescent="0.25">
@@ -6236,10 +6237,10 @@
         <v>571</v>
       </c>
       <c r="C288" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D288" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="289" spans="1:4" x14ac:dyDescent="0.25">
@@ -6250,10 +6251,10 @@
         <v>573</v>
       </c>
       <c r="C289" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D289" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="290" spans="1:4" x14ac:dyDescent="0.25">
@@ -6264,10 +6265,10 @@
         <v>575</v>
       </c>
       <c r="C290" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D290" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="291" spans="1:4" x14ac:dyDescent="0.25">
@@ -6278,7 +6279,7 @@
         <v>577</v>
       </c>
       <c r="C291" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D291" s="5">
         <v>0</v>
@@ -6292,7 +6293,7 @@
         <v>579</v>
       </c>
       <c r="C292" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D292" s="5">
         <v>0</v>
@@ -6306,7 +6307,7 @@
         <v>581</v>
       </c>
       <c r="C293" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D293" s="5">
         <v>0</v>
@@ -6320,7 +6321,7 @@
         <v>583</v>
       </c>
       <c r="C294" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D294" s="5">
         <v>0</v>
@@ -6334,7 +6335,7 @@
         <v>585</v>
       </c>
       <c r="C295" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D295" s="5">
         <v>0</v>
@@ -6348,7 +6349,7 @@
         <v>587</v>
       </c>
       <c r="C296" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D296" s="5">
         <v>0</v>
@@ -6362,7 +6363,7 @@
         <v>589</v>
       </c>
       <c r="C297" s="4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D297" s="5">
         <v>0</v>
@@ -6379,7 +6380,7 @@
         <v>0.7</v>
       </c>
       <c r="D298" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="299" spans="1:4" x14ac:dyDescent="0.25">
@@ -6393,7 +6394,7 @@
         <v>0.7</v>
       </c>
       <c r="D299" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="300" spans="1:4" x14ac:dyDescent="0.25">
@@ -6407,7 +6408,7 @@
         <v>0.7</v>
       </c>
       <c r="D300" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="301" spans="1:4" x14ac:dyDescent="0.25">
@@ -6417,8 +6418,12 @@
       <c r="B301" t="s">
         <v>597</v>
       </c>
-      <c r="C301" s="4"/>
-      <c r="D301" s="5"/>
+      <c r="C301" s="4">
+        <v>0.7</v>
+      </c>
+      <c r="D301" s="5">
+        <v>0</v>
+      </c>
     </row>
     <row r="302" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A302" t="s">
@@ -6427,8 +6432,12 @@
       <c r="B302" t="s">
         <v>599</v>
       </c>
-      <c r="C302" s="4"/>
-      <c r="D302" s="5"/>
+      <c r="C302" s="4">
+        <v>0.7</v>
+      </c>
+      <c r="D302" s="5">
+        <v>0</v>
+      </c>
     </row>
     <row r="303" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A303" t="s">
@@ -6438,11 +6447,10 @@
         <v>601</v>
       </c>
       <c r="C303" s="4">
-        <f>1/3</f>
-        <v>0.33333333333333331</v>
+        <v>0.7</v>
       </c>
       <c r="D303" s="5">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>